<commit_message>
After generalizing Review Documents method
</commit_message>
<xml_diff>
--- a/Data/Hires/testDataSlovakia.xlsx
+++ b/Data/Hires/testDataSlovakia.xlsx
@@ -1,35 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{016A5FAB-AF6F-4325-B3DF-503379EDD3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="222">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -334,7 +319,7 @@
     <t>SK Monthly</t>
   </si>
   <si>
-    <t>Meal Voucher Card </t>
+    <t xml:space="preserve">Meal Voucher Card </t>
   </si>
   <si>
     <t>Všeobecná zdrav. Poisť.</t>
@@ -500,7 +485,7 @@
     <t>Leffler</t>
   </si>
   <si>
-    <t>In-Store P&amp;C Supervisor_NEW  </t>
+    <t xml:space="preserve">In-Store P&amp;C Supervisor_NEW  </t>
   </si>
   <si>
     <t>Married (Slovakia)</t>
@@ -686,7 +671,10 @@
     <t>10651792</t>
   </si>
   <si>
-    <t>Caterina</t>
+    <t>Alexandria</t>
+  </si>
+  <si>
+    <t>Welch-Becker</t>
   </si>
   <si>
     <t>08 Ladieswear</t>
@@ -698,43 +686,43 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="2"/>
       <sz val="14"/>
-      <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -746,7 +734,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -757,7 +745,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -783,27 +771,17 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -813,25 +791,15 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -842,9 +810,7 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -854,38 +820,24 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top style="thin"/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <left style="thin"/>
+      <right style="thin"/>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1319,9 +1271,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CH36"/>
-  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -1411,7 +1363,7 @@
     <col min="87" max="87" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:86" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.5" customHeight="1" spans="1:86" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1649,7 +1601,7 @@
       <c r="CG1" s="11"/>
       <c r="CH1" s="12"/>
     </row>
-    <row r="2" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>72</v>
       </c>
@@ -1717,7 +1669,7 @@
         <v>81</v>
       </c>
       <c r="W2" s="21">
-        <f t="shared" ref="W2:W16" ca="1" si="0">TODAY()-31</f>
+        <f t="shared" ref="W2:W16" si="0">TODAY()-31</f>
         <v>45562</v>
       </c>
       <c r="X2" s="18" t="s">
@@ -1754,7 +1706,7 @@
         <v>95</v>
       </c>
       <c r="AI2" s="21">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>45958</v>
       </c>
       <c r="AJ2" s="18" t="s">
@@ -1809,7 +1761,7 @@
         <v>105</v>
       </c>
       <c r="BA2" s="19">
-        <f t="shared" ref="BA2:BA16" ca="1" si="1">TODAY()+90</f>
+        <f t="shared" ref="BA2:BA16" si="1">TODAY()+90</f>
         <v>45683</v>
       </c>
       <c r="BB2" s="15" t="s">
@@ -1825,15 +1777,15 @@
         <v>109</v>
       </c>
       <c r="BF2" s="19">
-        <f t="shared" ref="BF2:BF16" ca="1" si="2">W2</f>
+        <f t="shared" ref="BF2:BF16" si="2">W2</f>
         <v>45562</v>
       </c>
       <c r="BG2" s="19">
-        <f t="shared" ref="BG2:BG16" ca="1" si="3">W2</f>
+        <f t="shared" ref="BG2:BG16" si="3">W2</f>
         <v>45562</v>
       </c>
       <c r="BH2" s="21">
-        <f t="shared" ref="BH2:BH16" ca="1" si="4">AI2</f>
+        <f t="shared" ref="BH2:BH16" si="4">AI2</f>
         <v>45958</v>
       </c>
       <c r="BI2" s="28" t="s">
@@ -1843,7 +1795,7 @@
         <v>110</v>
       </c>
       <c r="BK2" s="30">
-        <f t="array" aca="1" ref="BK2:BK16" ca="1">_xlfn.RANDARRAY(15,1,1234567890,9999999999,TRUE)</f>
+        <f t="array" ref="BK2:BK16">_xlfn.RANDARRAY(15,1,1234567890,9999999999,TRUE)</f>
         <v>7028996362</v>
       </c>
       <c r="BL2" s="31" t="s">
@@ -1894,7 +1846,7 @@
       <c r="CG2" s="33"/>
       <c r="CH2" s="33"/>
     </row>
-    <row r="3" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>121</v>
       </c>
@@ -1962,7 +1914,7 @@
         <v>81</v>
       </c>
       <c r="W3" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X3" s="18" t="s">
@@ -2053,7 +2005,7 @@
         <v>82</v>
       </c>
       <c r="BA3" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB3" s="15" t="s">
@@ -2069,16 +2021,16 @@
         <v>109</v>
       </c>
       <c r="BF3" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG3" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
-      <c r="BH3" s="21" t="str">
+      <c r="BH3" s="21">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="BI3" s="28" t="s">
         <v>76</v>
@@ -2087,7 +2039,6 @@
         <v>110</v>
       </c>
       <c r="BK3" s="36">
-        <f ca="1"/>
         <v>3972936630</v>
       </c>
       <c r="BL3" s="31" t="s">
@@ -2138,7 +2089,7 @@
       <c r="CG3" s="33"/>
       <c r="CH3" s="33"/>
     </row>
-    <row r="4" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>136</v>
       </c>
@@ -2206,7 +2157,7 @@
         <v>81</v>
       </c>
       <c r="W4" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X4" s="18" t="s">
@@ -2243,7 +2194,7 @@
         <v>95</v>
       </c>
       <c r="AI4" s="21">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>45958</v>
       </c>
       <c r="AJ4" s="18" t="s">
@@ -2298,7 +2249,7 @@
         <v>82</v>
       </c>
       <c r="BA4" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB4" s="15" t="s">
@@ -2314,15 +2265,15 @@
         <v>109</v>
       </c>
       <c r="BF4" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG4" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH4" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45958</v>
       </c>
       <c r="BI4" s="28" t="s">
@@ -2332,7 +2283,6 @@
         <v>110</v>
       </c>
       <c r="BK4" s="36">
-        <f ca="1"/>
         <v>8861087480</v>
       </c>
       <c r="BL4" s="31" t="s">
@@ -2383,7 +2333,7 @@
       <c r="CG4" s="33"/>
       <c r="CH4" s="33"/>
     </row>
-    <row r="5" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>144</v>
       </c>
@@ -2451,7 +2401,7 @@
         <v>81</v>
       </c>
       <c r="W5" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X5" s="18" t="s">
@@ -2542,7 +2492,7 @@
         <v>82</v>
       </c>
       <c r="BA5" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB5" s="15" t="s">
@@ -2558,16 +2508,16 @@
         <v>109</v>
       </c>
       <c r="BF5" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG5" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
-      <c r="BH5" s="21" t="str">
+      <c r="BH5" s="21">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="BI5" s="28" t="s">
         <v>76</v>
@@ -2576,7 +2526,6 @@
         <v>110</v>
       </c>
       <c r="BK5" s="36">
-        <f ca="1"/>
         <v>7997866835</v>
       </c>
       <c r="BL5" s="31" t="s">
@@ -2627,7 +2576,7 @@
       <c r="CG5" s="33"/>
       <c r="CH5" s="33"/>
     </row>
-    <row r="6" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>152</v>
       </c>
@@ -2695,7 +2644,7 @@
         <v>81</v>
       </c>
       <c r="W6" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X6" s="18" t="s">
@@ -2732,7 +2681,7 @@
         <v>95</v>
       </c>
       <c r="AI6" s="21">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>45958</v>
       </c>
       <c r="AJ6" s="18" t="s">
@@ -2787,7 +2736,7 @@
         <v>82</v>
       </c>
       <c r="BA6" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB6" s="15" t="s">
@@ -2803,15 +2752,15 @@
         <v>109</v>
       </c>
       <c r="BF6" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG6" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH6" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45958</v>
       </c>
       <c r="BI6" s="28" t="s">
@@ -2821,7 +2770,6 @@
         <v>110</v>
       </c>
       <c r="BK6" s="36">
-        <f ca="1"/>
         <v>6720885372</v>
       </c>
       <c r="BL6" s="31" t="s">
@@ -2872,7 +2820,7 @@
       <c r="CG6" s="33"/>
       <c r="CH6" s="33"/>
     </row>
-    <row r="7" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>159</v>
       </c>
@@ -2940,7 +2888,7 @@
         <v>81</v>
       </c>
       <c r="W7" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X7" s="18" t="s">
@@ -3031,7 +2979,7 @@
         <v>82</v>
       </c>
       <c r="BA7" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB7" s="15" t="s">
@@ -3047,16 +2995,16 @@
         <v>109</v>
       </c>
       <c r="BF7" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG7" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
-      <c r="BH7" s="21" t="str">
+      <c r="BH7" s="21">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="BI7" s="28" t="s">
         <v>76</v>
@@ -3065,7 +3013,6 @@
         <v>110</v>
       </c>
       <c r="BK7" s="36">
-        <f ca="1"/>
         <v>2755314927</v>
       </c>
       <c r="BL7" s="31" t="s">
@@ -3116,7 +3063,7 @@
       <c r="CG7" s="33"/>
       <c r="CH7" s="33"/>
     </row>
-    <row r="8" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>165</v>
       </c>
@@ -3184,7 +3131,7 @@
         <v>81</v>
       </c>
       <c r="W8" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X8" s="18" t="s">
@@ -3221,7 +3168,7 @@
         <v>95</v>
       </c>
       <c r="AI8" s="21">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>45958</v>
       </c>
       <c r="AJ8" s="18" t="s">
@@ -3276,7 +3223,7 @@
         <v>82</v>
       </c>
       <c r="BA8" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB8" s="15" t="s">
@@ -3292,15 +3239,15 @@
         <v>109</v>
       </c>
       <c r="BF8" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG8" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH8" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45958</v>
       </c>
       <c r="BI8" s="28" t="s">
@@ -3310,7 +3257,6 @@
         <v>110</v>
       </c>
       <c r="BK8" s="36">
-        <f ca="1"/>
         <v>1778990826</v>
       </c>
       <c r="BL8" s="31" t="s">
@@ -3361,7 +3307,7 @@
       <c r="CG8" s="33"/>
       <c r="CH8" s="33"/>
     </row>
-    <row r="9" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>171</v>
       </c>
@@ -3429,7 +3375,7 @@
         <v>81</v>
       </c>
       <c r="W9" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X9" s="18" t="s">
@@ -3520,7 +3466,7 @@
         <v>105</v>
       </c>
       <c r="BA9" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB9" s="15" t="s">
@@ -3536,16 +3482,16 @@
         <v>109</v>
       </c>
       <c r="BF9" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG9" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
-      <c r="BH9" s="21" t="str">
+      <c r="BH9" s="21">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="BI9" s="28" t="s">
         <v>76</v>
@@ -3554,7 +3500,6 @@
         <v>110</v>
       </c>
       <c r="BK9" s="36">
-        <f ca="1"/>
         <v>8754468577</v>
       </c>
       <c r="BL9" s="31" t="s">
@@ -3605,7 +3550,7 @@
       <c r="CG9" s="33"/>
       <c r="CH9" s="33"/>
     </row>
-    <row r="10" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>177</v>
       </c>
@@ -3673,7 +3618,7 @@
         <v>81</v>
       </c>
       <c r="W10" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X10" s="18" t="s">
@@ -3710,7 +3655,7 @@
         <v>95</v>
       </c>
       <c r="AI10" s="21">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>45958</v>
       </c>
       <c r="AJ10" s="18" t="s">
@@ -3765,7 +3710,7 @@
         <v>82</v>
       </c>
       <c r="BA10" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB10" s="15" t="s">
@@ -3781,15 +3726,15 @@
         <v>109</v>
       </c>
       <c r="BF10" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG10" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH10" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45958</v>
       </c>
       <c r="BI10" s="28" t="s">
@@ -3799,7 +3744,6 @@
         <v>110</v>
       </c>
       <c r="BK10" s="36">
-        <f ca="1"/>
         <v>7796695246</v>
       </c>
       <c r="BL10" s="31" t="s">
@@ -3850,7 +3794,7 @@
       <c r="CG10" s="33"/>
       <c r="CH10" s="33"/>
     </row>
-    <row r="11" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>183</v>
       </c>
@@ -3918,7 +3862,7 @@
         <v>81</v>
       </c>
       <c r="W11" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X11" s="18" t="s">
@@ -4009,7 +3953,7 @@
         <v>82</v>
       </c>
       <c r="BA11" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB11" s="15" t="s">
@@ -4025,16 +3969,16 @@
         <v>109</v>
       </c>
       <c r="BF11" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG11" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
-      <c r="BH11" s="21" t="str">
+      <c r="BH11" s="21">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="BI11" s="28" t="s">
         <v>76</v>
@@ -4043,7 +3987,6 @@
         <v>110</v>
       </c>
       <c r="BK11" s="36">
-        <f ca="1"/>
         <v>6164841195</v>
       </c>
       <c r="BL11" s="31" t="s">
@@ -4094,7 +4037,7 @@
       <c r="CG11" s="33"/>
       <c r="CH11" s="33"/>
     </row>
-    <row r="12" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>189</v>
       </c>
@@ -4162,7 +4105,7 @@
         <v>81</v>
       </c>
       <c r="W12" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X12" s="18" t="s">
@@ -4199,7 +4142,7 @@
         <v>95</v>
       </c>
       <c r="AI12" s="21">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>45958</v>
       </c>
       <c r="AJ12" s="18" t="s">
@@ -4254,7 +4197,7 @@
         <v>82</v>
       </c>
       <c r="BA12" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB12" s="15" t="s">
@@ -4270,15 +4213,15 @@
         <v>109</v>
       </c>
       <c r="BF12" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG12" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH12" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45958</v>
       </c>
       <c r="BI12" s="28" t="s">
@@ -4288,7 +4231,6 @@
         <v>110</v>
       </c>
       <c r="BK12" s="36">
-        <f ca="1"/>
         <v>8855925579</v>
       </c>
       <c r="BL12" s="31" t="s">
@@ -4339,7 +4281,7 @@
       <c r="CG12" s="33"/>
       <c r="CH12" s="33"/>
     </row>
-    <row r="13" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>195</v>
       </c>
@@ -4407,7 +4349,7 @@
         <v>81</v>
       </c>
       <c r="W13" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X13" s="18" t="s">
@@ -4444,7 +4386,7 @@
         <v>95</v>
       </c>
       <c r="AI13" s="21">
-        <f ca="1">W13+360</f>
+        <f>W13+360</f>
         <v>45922</v>
       </c>
       <c r="AJ13" s="18" t="s">
@@ -4499,7 +4441,7 @@
         <v>82</v>
       </c>
       <c r="BA13" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB13" s="15" t="s">
@@ -4515,15 +4457,15 @@
         <v>109</v>
       </c>
       <c r="BF13" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG13" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH13" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45922</v>
       </c>
       <c r="BI13" s="28" t="s">
@@ -4533,7 +4475,6 @@
         <v>110</v>
       </c>
       <c r="BK13" s="36">
-        <f ca="1"/>
         <v>4776368626</v>
       </c>
       <c r="BL13" s="31" t="s">
@@ -4584,7 +4525,7 @@
       <c r="CG13" s="33"/>
       <c r="CH13" s="33"/>
     </row>
-    <row r="14" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>204</v>
       </c>
@@ -4652,7 +4593,7 @@
         <v>81</v>
       </c>
       <c r="W14" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X14" s="18" t="s">
@@ -4689,7 +4630,7 @@
         <v>95</v>
       </c>
       <c r="AI14" s="21">
-        <f ca="1">W14+365</f>
+        <f>W14+365</f>
         <v>45927</v>
       </c>
       <c r="AJ14" s="18" t="s">
@@ -4744,7 +4685,7 @@
         <v>105</v>
       </c>
       <c r="BA14" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB14" s="15" t="s">
@@ -4760,15 +4701,15 @@
         <v>109</v>
       </c>
       <c r="BF14" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG14" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH14" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45927</v>
       </c>
       <c r="BI14" s="28" t="s">
@@ -4778,7 +4719,6 @@
         <v>110</v>
       </c>
       <c r="BK14" s="36">
-        <f ca="1"/>
         <v>2310642433</v>
       </c>
       <c r="BL14" s="31" t="s">
@@ -4829,7 +4769,7 @@
       <c r="CG14" s="33"/>
       <c r="CH14" s="33"/>
     </row>
-    <row r="15" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>210</v>
       </c>
@@ -4897,7 +4837,7 @@
         <v>81</v>
       </c>
       <c r="W15" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X15" s="18" t="s">
@@ -4988,7 +4928,7 @@
         <v>82</v>
       </c>
       <c r="BA15" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB15" s="15" t="s">
@@ -5004,16 +4944,16 @@
         <v>109</v>
       </c>
       <c r="BF15" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG15" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
-      <c r="BH15" s="21" t="str">
+      <c r="BH15" s="21">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="BI15" s="28" t="s">
         <v>76</v>
@@ -5022,7 +4962,6 @@
         <v>110</v>
       </c>
       <c r="BK15" s="36">
-        <f ca="1"/>
         <v>3471633201</v>
       </c>
       <c r="BL15" s="31" t="s">
@@ -5073,7 +5012,7 @@
       <c r="CG15" s="33"/>
       <c r="CH15" s="33"/>
     </row>
-    <row r="16" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>216</v>
       </c>
@@ -5093,7 +5032,7 @@
         <v>218</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>168</v>
+        <v>219</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>79</v>
@@ -5141,7 +5080,7 @@
         <v>81</v>
       </c>
       <c r="W16" s="21">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45562</v>
       </c>
       <c r="X16" s="18" t="s">
@@ -5178,7 +5117,7 @@
         <v>95</v>
       </c>
       <c r="AI16" s="21">
-        <f ca="1">W16+360</f>
+        <f>W16+360</f>
         <v>45922</v>
       </c>
       <c r="AJ16" s="18" t="s">
@@ -5188,7 +5127,7 @@
         <v>97</v>
       </c>
       <c r="AL16" s="38" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AM16" s="18" t="s">
         <v>99</v>
@@ -5233,11 +5172,11 @@
         <v>82</v>
       </c>
       <c r="BA16" s="19">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45683</v>
       </c>
       <c r="BB16" s="15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="BC16" s="18" t="s">
         <v>107</v>
@@ -5249,15 +5188,15 @@
         <v>109</v>
       </c>
       <c r="BF16" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45562</v>
       </c>
       <c r="BG16" s="19">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45562</v>
       </c>
       <c r="BH16" s="21">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45922</v>
       </c>
       <c r="BI16" s="28" t="s">
@@ -5267,7 +5206,6 @@
         <v>110</v>
       </c>
       <c r="BK16" s="39">
-        <f ca="1"/>
         <v>2444594880</v>
       </c>
       <c r="BL16" s="31" t="s">
@@ -5318,7 +5256,7 @@
       <c r="CG16" s="33"/>
       <c r="CH16" s="33"/>
     </row>
-    <row r="17" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.65" customHeight="1" spans="2:86" x14ac:dyDescent="0.25">
       <c r="B17" s="35"/>
       <c r="E17" s="35"/>
       <c r="G17" s="14"/>
@@ -5401,7 +5339,7 @@
       <c r="CG17" s="33"/>
       <c r="CH17" s="33"/>
     </row>
-    <row r="18" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G18" s="14"/>
       <c r="H18" s="40"/>
       <c r="I18" s="37"/>
@@ -5481,7 +5419,7 @@
       <c r="CG18" s="33"/>
       <c r="CH18" s="33"/>
     </row>
-    <row r="19" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G19" s="14"/>
       <c r="H19" s="40"/>
       <c r="I19" s="37"/>
@@ -5561,7 +5499,7 @@
       <c r="CG19" s="33"/>
       <c r="CH19" s="33"/>
     </row>
-    <row r="20" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G20" s="14"/>
       <c r="H20" s="40"/>
       <c r="I20" s="37"/>
@@ -5641,7 +5579,7 @@
       <c r="CG20" s="33"/>
       <c r="CH20" s="33"/>
     </row>
-    <row r="21" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G21" s="14"/>
       <c r="H21" s="40"/>
       <c r="I21" s="37"/>
@@ -5721,7 +5659,7 @@
       <c r="CG21" s="33"/>
       <c r="CH21" s="33"/>
     </row>
-    <row r="22" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G22" s="14"/>
       <c r="H22" s="40"/>
       <c r="I22" s="37"/>
@@ -5801,7 +5739,7 @@
       <c r="CG22" s="33"/>
       <c r="CH22" s="33"/>
     </row>
-    <row r="23" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G23" s="14"/>
       <c r="H23" s="40"/>
       <c r="I23" s="37"/>
@@ -5881,7 +5819,7 @@
       <c r="CG23" s="33"/>
       <c r="CH23" s="33"/>
     </row>
-    <row r="24" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G24" s="14"/>
       <c r="H24" s="40"/>
       <c r="I24" s="37"/>
@@ -5961,7 +5899,7 @@
       <c r="CG24" s="33"/>
       <c r="CH24" s="33"/>
     </row>
-    <row r="25" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G25" s="14"/>
       <c r="H25" s="40"/>
       <c r="I25" s="37"/>
@@ -6041,7 +5979,7 @@
       <c r="CG25" s="33"/>
       <c r="CH25" s="33"/>
     </row>
-    <row r="26" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G26" s="14"/>
       <c r="H26" s="40"/>
       <c r="I26" s="37"/>
@@ -6121,7 +6059,7 @@
       <c r="CG26" s="33"/>
       <c r="CH26" s="33"/>
     </row>
-    <row r="27" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G27" s="14"/>
       <c r="H27" s="40"/>
       <c r="I27" s="37"/>
@@ -6201,7 +6139,7 @@
       <c r="CG27" s="33"/>
       <c r="CH27" s="33"/>
     </row>
-    <row r="28" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G28" s="14"/>
       <c r="H28" s="40"/>
       <c r="I28" s="37"/>
@@ -6281,7 +6219,7 @@
       <c r="CG28" s="33"/>
       <c r="CH28" s="33"/>
     </row>
-    <row r="29" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G29" s="14"/>
       <c r="H29" s="40"/>
       <c r="I29" s="37"/>
@@ -6361,7 +6299,7 @@
       <c r="CG29" s="33"/>
       <c r="CH29" s="33"/>
     </row>
-    <row r="30" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G30" s="14"/>
       <c r="H30" s="40"/>
       <c r="I30" s="37"/>
@@ -6441,7 +6379,7 @@
       <c r="CG30" s="33"/>
       <c r="CH30" s="33"/>
     </row>
-    <row r="31" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G31" s="14"/>
       <c r="H31" s="40"/>
       <c r="I31" s="37"/>
@@ -6521,7 +6459,7 @@
       <c r="CG31" s="33"/>
       <c r="CH31" s="33"/>
     </row>
-    <row r="32" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G32" s="14"/>
       <c r="H32" s="40"/>
       <c r="I32" s="37"/>
@@ -6601,7 +6539,7 @@
       <c r="CG32" s="33"/>
       <c r="CH32" s="33"/>
     </row>
-    <row r="33" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G33" s="14"/>
       <c r="H33" s="40"/>
       <c r="I33" s="37"/>
@@ -6681,7 +6619,7 @@
       <c r="CG33" s="33"/>
       <c r="CH33" s="33"/>
     </row>
-    <row r="34" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G34" s="14"/>
       <c r="H34" s="40"/>
       <c r="I34" s="37"/>
@@ -6762,7 +6700,7 @@
       <c r="CG34" s="33"/>
       <c r="CH34" s="33"/>
     </row>
-    <row r="35" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" ht="15.65" customHeight="1" spans="7:86" x14ac:dyDescent="0.25">
       <c r="G35" s="14"/>
       <c r="H35" s="40"/>
       <c r="I35" s="37"/>
@@ -6843,7 +6781,7 @@
       <c r="CG35" s="33"/>
       <c r="CH35" s="33"/>
     </row>
-    <row r="36" spans="2:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" ht="15.65" customHeight="1" spans="2:86" x14ac:dyDescent="0.25">
       <c r="B36" s="35"/>
       <c r="E36" s="35"/>
       <c r="G36" s="14"/>
@@ -6927,54 +6865,111 @@
       <c r="CH36" s="33"/>
     </row>
   </sheetData>
-  <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA17:AA36 Y17:Y36 BB17:BB36" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="28">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA17:AA36">
       <formula1>INDIRECT($H2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE10:BE16 X10:X16 V10:V36 S10:S16 J10:J16 CB10:CB36 BU10:BU16" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BB17:BB36">
       <formula1>INDIRECT($H2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2:BE16 X2:X16 V2:V36 S2:S16 J2:J16 CB2:CB36 BU2:BU16" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE10:BE16">
       <formula1>INDIRECT($H2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L17:L20 M19:M20 M17 L33:M34 L28:M31 L23:M25" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2:BE16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU10:BU16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB10:CB36">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB36">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J10:J16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L17:L20">
       <formula1>INDIRECT(#REF!)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L21:M22" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L21:M22">
       <formula1>INDIRECT($H3)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L26:M27" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L23:M25">
+      <formula1>INDIRECT(#REF!)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L26:M27">
       <formula1>INDIRECT($H5)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L32:M32" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L28:M31">
+      <formula1>INDIRECT(#REF!)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L32:M32">
       <formula1>INDIRECT($H7)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L35:M36" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L33:M34">
+      <formula1>INDIRECT(#REF!)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L35:M36">
       <formula1>INDIRECT($H8)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M18" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M17">
+      <formula1>INDIRECT(#REF!)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M18">
       <formula1>INDIRECT($H8)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M19:M20">
+      <formula1>INDIRECT(#REF!)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S10:S16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V36">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V36">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X10:X16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X16">
+      <formula1>INDIRECT($H2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y17:Y36">
+      <formula1>INDIRECT($H2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="U4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="U5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="U6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="U7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="U8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="U9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="U10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="U11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="U12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="U13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="U14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="U15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="U16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="U2" r:id="rId1"/>
+    <hyperlink ref="U3" r:id="rId2"/>
+    <hyperlink ref="U4" r:id="rId3"/>
+    <hyperlink ref="U5" r:id="rId4"/>
+    <hyperlink ref="U6" r:id="rId5"/>
+    <hyperlink ref="U7" r:id="rId6"/>
+    <hyperlink ref="U8" r:id="rId7"/>
+    <hyperlink ref="U9" r:id="rId8"/>
+    <hyperlink ref="U10" r:id="rId9"/>
+    <hyperlink ref="U11" r:id="rId10"/>
+    <hyperlink ref="U12" r:id="rId11"/>
+    <hyperlink ref="U13" r:id="rId12"/>
+    <hyperlink ref="U14" r:id="rId13"/>
+    <hyperlink ref="U15" r:id="rId14"/>
+    <hyperlink ref="U16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>